<commit_message>
Ablation Study update and small updates for PV and Timestamp models
</commit_message>
<xml_diff>
--- a/Ablation_Study/data/cnn_modality_outputs/cnn_modality_summary.xlsx
+++ b/Ablation_Study/data/cnn_modality_outputs/cnn_modality_summary.xlsx
@@ -528,46 +528,46 @@
         <v>51</v>
       </c>
       <c r="D2" t="n">
-        <v>2.743381500244141</v>
+        <v>4.804327487945557</v>
       </c>
       <c r="E2" t="n">
-        <v>3.445594412759396</v>
+        <v>5.996393073249619</v>
       </c>
       <c r="F2" t="n">
-        <v>3.467229604721069</v>
+        <v>6.555027008056641</v>
       </c>
       <c r="G2" t="n">
-        <v>4.292648844995979</v>
+        <v>7.444696615069662</v>
       </c>
       <c r="H2" t="n">
-        <v>3.889603853225708</v>
+        <v>9.06661319732666</v>
       </c>
       <c r="I2" t="n">
-        <v>4.312102368585212</v>
+        <v>9.512917018977982</v>
       </c>
       <c r="J2" t="n">
-        <v>4.003793716430664</v>
+        <v>5.883502960205078</v>
       </c>
       <c r="K2" t="n">
-        <v>4.503761414898021</v>
+        <v>6.593256493491274</v>
       </c>
       <c r="L2" t="n">
-        <v>2.027521133422852</v>
+        <v>3.229470491409302</v>
       </c>
       <c r="M2" t="n">
-        <v>2.613510418296237</v>
+        <v>3.803440148015174</v>
       </c>
       <c r="N2" t="n">
-        <v>1.905135154724121</v>
+        <v>2.151313066482544</v>
       </c>
       <c r="O2" t="n">
-        <v>2.224281400730085</v>
+        <v>2.52817810530934</v>
       </c>
       <c r="P2" t="n">
-        <v>1.167006254196167</v>
+        <v>1.940037965774536</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.466265504694896</v>
+        <v>2.343588251254571</v>
       </c>
     </row>
     <row r="3">
@@ -583,46 +583,46 @@
         <v>51</v>
       </c>
       <c r="D3" t="n">
-        <v>3.695486068725586</v>
+        <v>5.266489505767822</v>
       </c>
       <c r="E3" t="n">
-        <v>4.936197229732652</v>
+        <v>7.01640685892437</v>
       </c>
       <c r="F3" t="n">
-        <v>7.00600004196167</v>
+        <v>9.513247489929199</v>
       </c>
       <c r="G3" t="n">
-        <v>8.31976734936492</v>
+        <v>11.01709909518583</v>
       </c>
       <c r="H3" t="n">
-        <v>4.338794708251953</v>
+        <v>7.254741668701172</v>
       </c>
       <c r="I3" t="n">
-        <v>5.122687585690342</v>
+        <v>8.368328568756604</v>
       </c>
       <c r="J3" t="n">
-        <v>2.788975954055786</v>
+        <v>4.797458171844482</v>
       </c>
       <c r="K3" t="n">
-        <v>3.757692584941888</v>
+        <v>6.144302781035377</v>
       </c>
       <c r="L3" t="n">
-        <v>3.316286087036133</v>
+        <v>6.040154933929443</v>
       </c>
       <c r="M3" t="n">
-        <v>4.334653042082983</v>
+        <v>7.299595850378116</v>
       </c>
       <c r="N3" t="n">
-        <v>2.788831472396851</v>
+        <v>2.297173500061035</v>
       </c>
       <c r="O3" t="n">
-        <v>3.519276261486598</v>
+        <v>2.84756817046996</v>
       </c>
       <c r="P3" t="n">
-        <v>1.934026002883911</v>
+        <v>1.696159482002258</v>
       </c>
       <c r="Q3" t="n">
-        <v>2.332601455166532</v>
+        <v>2.197525809248213</v>
       </c>
     </row>
     <row r="4">
@@ -638,46 +638,46 @@
         <v>51</v>
       </c>
       <c r="D4" t="n">
-        <v>4.104476451873779</v>
+        <v>4.366806507110596</v>
       </c>
       <c r="E4" t="n">
-        <v>5.681059827653715</v>
+        <v>7.385926767514547</v>
       </c>
       <c r="F4" t="n">
-        <v>6.203522205352783</v>
+        <v>8.607087135314941</v>
       </c>
       <c r="G4" t="n">
-        <v>7.815819363196365</v>
+        <v>13.40323460952791</v>
       </c>
       <c r="H4" t="n">
-        <v>5.99617862701416</v>
+        <v>5.420159816741943</v>
       </c>
       <c r="I4" t="n">
-        <v>7.159749736994074</v>
+        <v>7.469545457689003</v>
       </c>
       <c r="J4" t="n">
-        <v>4.014102935791016</v>
+        <v>3.8657066822052</v>
       </c>
       <c r="K4" t="n">
-        <v>6.01162769231315</v>
+        <v>6.458486772580831</v>
       </c>
       <c r="L4" t="n">
-        <v>4.231477737426758</v>
+        <v>4.53620719909668</v>
       </c>
       <c r="M4" t="n">
-        <v>5.67419184505445</v>
+        <v>6.222137295430997</v>
       </c>
       <c r="N4" t="n">
-        <v>2.333981275558472</v>
+        <v>2.371341943740845</v>
       </c>
       <c r="O4" t="n">
-        <v>2.834556053965292</v>
+        <v>2.917287070276566</v>
       </c>
       <c r="P4" t="n">
-        <v>1.84759247303009</v>
+        <v>1.400337815284729</v>
       </c>
       <c r="Q4" t="n">
-        <v>2.219628066274617</v>
+        <v>1.712647023816068</v>
       </c>
     </row>
   </sheetData>

</xml_diff>